<commit_message>
Add directional skill hit contracts
</commit_message>
<xml_diff>
--- a/ExcelTable/Character.xlsx
+++ b/ExcelTable/Character.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="1" r:id="R5e717dcce3984124"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="1" r:id="R1f86af1539974d38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51,12 +51,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -104,7 +129,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -156,6 +181,19 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -394,6 +432,7 @@
     <x:col min="17" max="17" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -454,6 +493,9 @@
       <x:c r="S1" s="7" t="str">
         <x:v>HitAnimationDurationSeconds</x:v>
       </x:c>
+      <x:c r="T1" s="20" t="str">
+        <x:v>BasicAttackSkillInfoIndex</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -513,6 +555,9 @@
       <x:c r="S2" s="9" t="str">
         <x:v>server</x:v>
       </x:c>
+      <x:c r="T2" s="22" t="str">
+        <x:v>server</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -572,6 +617,9 @@
       <x:c r="S3" s="12" t="str">
         <x:v>피격 행동을 잠그고 피격 애니메이션을 유지하는 시간입니다.</x:v>
       </x:c>
+      <x:c r="T3" s="25" t="str">
+        <x:v>Skill.xlsx/SkillInfo의 기본 공격 행 인덱스입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -631,6 +679,9 @@
       <x:c r="S4" s="14" t="str">
         <x:v>float</x:v>
       </x:c>
+      <x:c r="T4" s="27" t="str">
+        <x:v>int</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -689,6 +740,9 @@
       </x:c>
       <x:c r="S5" s="17" t="n">
         <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="T5" s="29" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Rebuild ladder climb state flow
</commit_message>
<xml_diff>
--- a/ExcelTable/Character.xlsx
+++ b/ExcelTable/Character.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="1" r:id="R1f86af1539974d38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="1" r:id="Raa0dafe84c104ffb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51,12 +51,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -129,7 +154,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -194,6 +219,19 @@
     <x:xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -433,6 +471,7 @@
     <x:col min="18" max="18" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="23.75" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18.1299991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -496,6 +535,9 @@
       <x:c r="T1" s="20" t="str">
         <x:v>BasicAttackSkillInfoIndex</x:v>
       </x:c>
+      <x:c r="U1" s="31" t="str">
+        <x:v>LadderClimbSpeed</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -558,6 +600,9 @@
       <x:c r="T2" s="22" t="str">
         <x:v>server</x:v>
       </x:c>
+      <x:c r="U2" s="33" t="str">
+        <x:v>server</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -620,6 +665,9 @@
       <x:c r="T3" s="25" t="str">
         <x:v>Skill.xlsx/SkillInfo의 기본 공격 행 인덱스입니다.</x:v>
       </x:c>
+      <x:c r="U3" s="36" t="str">
+        <x:v>사다리 탑승 중 초당 세계 Y 이동 속도입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -682,6 +730,9 @@
       <x:c r="T4" s="27" t="str">
         <x:v>int</x:v>
       </x:c>
+      <x:c r="U4" s="38" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -742,6 +793,9 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="T5" s="29" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U5" s="40" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Fix combat action priority and ladder climb
</commit_message>
<xml_diff>
--- a/ExcelTable/Character.xlsx
+++ b/ExcelTable/Character.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="1" r:id="Raa0dafe84c104ffb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PlayerStatsProfiles" sheetId="1" r:id="R113b7bd5ea094b0b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51,12 +51,37 @@
       <x:name val="Malgun Gothic"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2E8F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -154,7 +179,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="52">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
@@ -232,6 +257,19 @@
     <x:xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -472,6 +510,7 @@
     <x:col min="19" max="19" width="18.1299991607666" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="23.75" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="18.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="23.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.5" customHeight="1">
@@ -538,6 +577,9 @@
       <x:c r="U1" s="31" t="str">
         <x:v>LadderClimbSpeed</x:v>
       </x:c>
+      <x:c r="V1" s="42" t="str">
+        <x:v>LadderExitStandOffset</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="16.5" customHeight="1">
       <x:c r="A2" s="9" t="str">
@@ -603,6 +645,9 @@
       <x:c r="U2" s="33" t="str">
         <x:v>server</x:v>
       </x:c>
+      <x:c r="V2" s="44" t="str">
+        <x:v>server</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="12" t="str">
@@ -668,6 +713,9 @@
       <x:c r="U3" s="36" t="str">
         <x:v>사다리 탑승 중 초당 세계 Y 이동 속도입니다.</x:v>
       </x:c>
+      <x:c r="V3" s="47" t="str">
+        <x:v>사다리에서 내릴 때 발판 표면보다 위로 이동할 Y 안착 오프셋입니다.</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="16.5" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -733,6 +781,9 @@
       <x:c r="U4" s="38" t="str">
         <x:v>float</x:v>
       </x:c>
+      <x:c r="V4" s="49" t="str">
+        <x:v>float</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="16.5" customHeight="1">
       <x:c r="A5" s="17" t="n">
@@ -797,6 +848,9 @@
       </x:c>
       <x:c r="U5" s="40" t="n">
         <x:v>1</x:v>
+      </x:c>
+      <x:c r="V5" s="51" t="n">
+        <x:v>0.08</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>